<commit_message>
feat: uploading everything on remote work pc, preparing for management changes.
</commit_message>
<xml_diff>
--- a/data_analisys/entries_cumsum.xlsx
+++ b/data_analisys/entries_cumsum.xlsx
@@ -380,7 +380,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -399,13 +399,13 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>2002</v>
+        <v>1997</v>
       </c>
       <c r="C2">
-        <v>83527</v>
+        <v>2873</v>
       </c>
       <c r="D2">
-        <v>83527</v>
+        <v>2873</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -413,13 +413,13 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2003</v>
+        <v>1998</v>
       </c>
       <c r="C3">
-        <v>138166</v>
+        <v>4187</v>
       </c>
       <c r="D3">
-        <v>221693</v>
+        <v>7060</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -427,13 +427,13 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2004</v>
+        <v>1999</v>
       </c>
       <c r="C4">
-        <v>240639</v>
+        <v>20497</v>
       </c>
       <c r="D4">
-        <v>462332</v>
+        <v>27557</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -441,13 +441,13 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>2005</v>
+        <v>2000</v>
       </c>
       <c r="C5">
-        <v>322645</v>
+        <v>58521</v>
       </c>
       <c r="D5">
-        <v>784977</v>
+        <v>86078</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -455,13 +455,13 @@
         <v>4</v>
       </c>
       <c r="B6">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="C6">
-        <v>358892</v>
+        <v>51306</v>
       </c>
       <c r="D6">
-        <v>1143869</v>
+        <v>137384</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -469,13 +469,13 @@
         <v>5</v>
       </c>
       <c r="B7">
-        <v>2007</v>
+        <v>2002</v>
       </c>
       <c r="C7">
-        <v>524776</v>
+        <v>83527</v>
       </c>
       <c r="D7">
-        <v>1668645</v>
+        <v>220911</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -483,13 +483,13 @@
         <v>6</v>
       </c>
       <c r="B8">
-        <v>2008</v>
+        <v>2003</v>
       </c>
       <c r="C8">
-        <v>627414</v>
+        <v>138166</v>
       </c>
       <c r="D8">
-        <v>2296059</v>
+        <v>359077</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -497,13 +497,13 @@
         <v>7</v>
       </c>
       <c r="B9">
-        <v>2009</v>
+        <v>2004</v>
       </c>
       <c r="C9">
-        <v>764074</v>
+        <v>240639</v>
       </c>
       <c r="D9">
-        <v>3060133</v>
+        <v>599716</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -511,13 +511,13 @@
         <v>8</v>
       </c>
       <c r="B10">
-        <v>2010</v>
+        <v>2005</v>
       </c>
       <c r="C10">
-        <v>1041136</v>
+        <v>322645</v>
       </c>
       <c r="D10">
-        <v>4101269</v>
+        <v>922361</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -525,13 +525,13 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>2011</v>
+        <v>2006</v>
       </c>
       <c r="C11">
-        <v>1272610</v>
+        <v>358892</v>
       </c>
       <c r="D11">
-        <v>5373879</v>
+        <v>1281253</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -539,13 +539,13 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>2012</v>
+        <v>2007</v>
       </c>
       <c r="C12">
-        <v>1211353</v>
+        <v>524776</v>
       </c>
       <c r="D12">
-        <v>6585232</v>
+        <v>1806029</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -553,13 +553,13 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>2013</v>
+        <v>2008</v>
       </c>
       <c r="C13">
-        <v>1322341</v>
+        <v>627414</v>
       </c>
       <c r="D13">
-        <v>7907573</v>
+        <v>2433443</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -567,13 +567,13 @@
         <v>12</v>
       </c>
       <c r="B14">
-        <v>2014</v>
+        <v>2009</v>
       </c>
       <c r="C14">
-        <v>1732048</v>
+        <v>764074</v>
       </c>
       <c r="D14">
-        <v>9639621</v>
+        <v>3197517</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -581,13 +581,13 @@
         <v>13</v>
       </c>
       <c r="B15">
-        <v>2015</v>
+        <v>2010</v>
       </c>
       <c r="C15">
-        <v>2010727</v>
+        <v>1041136</v>
       </c>
       <c r="D15">
-        <v>11650348</v>
+        <v>4238653</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -595,13 +595,13 @@
         <v>14</v>
       </c>
       <c r="B16">
-        <v>2016</v>
+        <v>2011</v>
       </c>
       <c r="C16">
-        <v>2035070</v>
+        <v>1300828</v>
       </c>
       <c r="D16">
-        <v>13685418</v>
+        <v>5539481</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -609,13 +609,13 @@
         <v>15</v>
       </c>
       <c r="B17">
-        <v>2017</v>
+        <v>2012</v>
       </c>
       <c r="C17">
-        <v>1908731</v>
+        <v>1231038</v>
       </c>
       <c r="D17">
-        <v>15594149</v>
+        <v>6770519</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -623,13 +623,13 @@
         <v>16</v>
       </c>
       <c r="B18">
-        <v>2018</v>
+        <v>2013</v>
       </c>
       <c r="C18">
-        <v>1707494</v>
+        <v>1322341</v>
       </c>
       <c r="D18">
-        <v>17301643</v>
+        <v>8092860</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -637,13 +637,13 @@
         <v>17</v>
       </c>
       <c r="B19">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="C19">
-        <v>1589068</v>
+        <v>1732048</v>
       </c>
       <c r="D19">
-        <v>18890711</v>
+        <v>9824908</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -651,13 +651,13 @@
         <v>18</v>
       </c>
       <c r="B20">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="C20">
-        <v>1721738</v>
+        <v>2010727</v>
       </c>
       <c r="D20">
-        <v>20612449</v>
+        <v>11835635</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -665,13 +665,13 @@
         <v>19</v>
       </c>
       <c r="B21">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="C21">
-        <v>1839779</v>
+        <v>2044815</v>
       </c>
       <c r="D21">
-        <v>22452228</v>
+        <v>13880450</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -679,13 +679,13 @@
         <v>20</v>
       </c>
       <c r="B22">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="C22">
-        <v>1656717</v>
+        <v>1952531</v>
       </c>
       <c r="D22">
-        <v>24108945</v>
+        <v>15832981</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -693,13 +693,13 @@
         <v>21</v>
       </c>
       <c r="B23">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="C23">
-        <v>1470565</v>
+        <v>1751294</v>
       </c>
       <c r="D23">
-        <v>25579510</v>
+        <v>17584275</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -707,13 +707,13 @@
         <v>22</v>
       </c>
       <c r="B24">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="C24">
-        <v>1267857</v>
+        <v>1623093</v>
       </c>
       <c r="D24">
-        <v>26847367</v>
+        <v>19207368</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -721,13 +721,55 @@
         <v>23</v>
       </c>
       <c r="B25">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="C25">
-        <v>420128</v>
+        <v>1711402</v>
       </c>
       <c r="D25">
-        <v>27267495</v>
+        <v>20918770</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="1">
+        <v>24</v>
+      </c>
+      <c r="B26">
+        <v>2021</v>
+      </c>
+      <c r="C26">
+        <v>1778614</v>
+      </c>
+      <c r="D26">
+        <v>22697384</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="1">
+        <v>25</v>
+      </c>
+      <c r="B27">
+        <v>2022</v>
+      </c>
+      <c r="C27">
+        <v>1597761</v>
+      </c>
+      <c r="D27">
+        <v>24295145</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="1">
+        <v>26</v>
+      </c>
+      <c r="B28">
+        <v>2023</v>
+      </c>
+      <c r="C28">
+        <v>1409620</v>
+      </c>
+      <c r="D28">
+        <v>25704765</v>
       </c>
     </row>
   </sheetData>

</xml_diff>